<commit_message>
2025.11.20 Taylor series, area 18w
</commit_message>
<xml_diff>
--- a/HW5/Softmax_table.xlsx
+++ b/HW5/Softmax_table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c1d8b65b6adf7979/桌面/Github File/IC_Design_Laboratory/HW5/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="230" documentId="11_1B85D0BDD370594FA3B82111595ED87656CB84C1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF52878F-A805-4B1E-A268-8FD1D9506C7C}"/>
+  <xr:revisionPtr revIDLastSave="455" documentId="11_1B85D0BDD370594FA3B82111595ED87656CB84C1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B55C661F-0CC7-4A37-923C-6625925A433E}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3108" uniqueCount="3092">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3145" uniqueCount="3125">
   <si>
     <t>Fixed-point Input (4Q6)</t>
   </si>
@@ -8832,9 +8832,6 @@
   </si>
   <si>
     <t>0.47236655274101480017634457908570766448974609375</t>
-  </si>
-  <si>
-    <t>531837457726680</t>
   </si>
   <si>
     <t>0.4798052435596775304390357660235938813242147370504269939226478799473997045225714644117531988220930455</t>
@@ -9325,6 +9322,142 @@
   </si>
   <si>
     <t>插值</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>1538472748139629</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>stage1</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>stage2</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>stage3</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>stage4</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>stage5</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>stage6</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>stage7</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>stage8</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>stage9</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>mul 1/24</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>add 1/6</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>mul (x-a)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>add 1/2</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>add 1</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> mul expa</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>2731*16</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;&lt;4</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;&lt;21</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>1*2^21</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>1*2^26</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;&lt;26</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>1*2^30</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;&lt;30</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>495312&lt;&lt;30</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>lut point a</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>dev</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>對齊小數點</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>exp(a)真值</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>exp(x)誤差</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>求 EXP(982)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>exp(a)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>exp(x)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>DATAFLOW設計: 這部分錯誤, 因為對其不是左移四位, 應為六位, 直接更新在code上</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -9333,12 +9466,12 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="6">
-    <numFmt numFmtId="195" formatCode="0.00_);[Red]\(0.00\)"/>
-    <numFmt numFmtId="197" formatCode="0_);[Red]\(0\)"/>
-    <numFmt numFmtId="200" formatCode="0.0000%"/>
-    <numFmt numFmtId="203" formatCode="0.0000000%"/>
-    <numFmt numFmtId="205" formatCode="0.0000000"/>
-    <numFmt numFmtId="206" formatCode="0.000000"/>
+    <numFmt numFmtId="176" formatCode="0.00_);[Red]\(0.00\)"/>
+    <numFmt numFmtId="177" formatCode="0_);[Red]\(0\)"/>
+    <numFmt numFmtId="178" formatCode="0.0000%"/>
+    <numFmt numFmtId="179" formatCode="0.0000000%"/>
+    <numFmt numFmtId="180" formatCode="0.0000000"/>
+    <numFmt numFmtId="181" formatCode="0.000000"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -9384,7 +9517,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -9444,6 +9577,15 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -9451,22 +9593,28 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="195" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="197" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="205" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="206" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="181" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -9774,7 +9922,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H1048"/>
+  <dimension ref="A1:H1073"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.19921875" bestFit="1" customWidth="1"/>
@@ -9783,12 +9931,12 @@
     <col min="4" max="4" width="27.8984375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="29.3984375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.8984375" customWidth="1"/>
-    <col min="7" max="7" width="11.8984375" customWidth="1"/>
+    <col min="7" max="7" width="49.8984375" customWidth="1"/>
     <col min="8" max="8" width="11.3984375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.69921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -9804,8 +9952,11 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G1" s="8" t="s">
+        <v>3091</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>0</v>
       </c>
@@ -9822,10 +9973,14 @@
         <v>6</v>
       </c>
       <c r="F2" t="s">
-        <v>3075</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+        <v>3074</v>
+      </c>
+      <c r="G2" s="2">
+        <f>E2-G1</f>
+        <v>-412572841297000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -9841,8 +9996,12 @@
       <c r="E3" s="3">
         <v>1143630250473350</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G3" s="2">
+        <f t="shared" ref="G3:G23" si="0">E3-G2</f>
+        <v>1556203091770350</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
@@ -9858,8 +10017,12 @@
       <c r="E4" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G4" s="2">
+        <f t="shared" si="0"/>
+        <v>-394563285381620</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
@@ -9875,8 +10038,12 @@
       <c r="E5" s="2" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G5" s="2">
+        <f t="shared" si="0"/>
+        <v>1574496256924050</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>4</v>
       </c>
@@ -9892,8 +10059,12 @@
       <c r="E6" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G6" s="2">
+        <f t="shared" si="0"/>
+        <v>-375982044793950</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>5</v>
       </c>
@@ -9909,8 +10080,12 @@
       <c r="E7" s="2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G7" s="2">
+        <f t="shared" si="0"/>
+        <v>1593370109473680</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>6</v>
       </c>
@@ -9926,8 +10101,12 @@
       <c r="E8" s="2" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G8" s="2">
+        <f t="shared" si="0"/>
+        <v>-356810972314470</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>7</v>
       </c>
@@ -9943,8 +10122,12 @@
       <c r="E9" s="2" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G9" s="2">
+        <f t="shared" si="0"/>
+        <v>1612843082415870</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>8</v>
       </c>
@@ -9960,8 +10143,12 @@
       <c r="E10" s="2" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G10" s="2">
+        <f t="shared" si="0"/>
+        <v>-337031344669070</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>9</v>
       </c>
@@ -9977,8 +10164,12 @@
       <c r="E11" s="2" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G11" s="2">
+        <f t="shared" si="0"/>
+        <v>1632934193873380</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>10</v>
       </c>
@@ -9994,8 +10185,12 @@
       <c r="E12" s="2" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G12" s="2">
+        <f t="shared" si="0"/>
+        <v>-316623844243150</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>11</v>
       </c>
@@ -10011,8 +10206,12 @@
       <c r="E13" s="2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G13" s="2">
+        <f t="shared" si="0"/>
+        <v>1653663065669000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>12</v>
       </c>
@@ -10028,8 +10227,12 @@
       <c r="E14" s="2" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G14" s="2">
+        <f t="shared" si="0"/>
+        <v>-295568540215170</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>13</v>
       </c>
@@ -10045,8 +10248,12 @@
       <c r="E15" s="2" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G15" s="2">
+        <f t="shared" si="0"/>
+        <v>1675049942489020</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>14</v>
       </c>
@@ -10062,8 +10269,12 @@
       <c r="E16" s="2" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G16" s="2">
+        <f t="shared" si="0"/>
+        <v>-273844869091410</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>15</v>
       </c>
@@ -10079,8 +10290,12 @@
       <c r="E17" s="2" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G17" s="2">
+        <f t="shared" si="0"/>
+        <v>1697115711655080</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>16</v>
       </c>
@@ -10096,8 +10311,12 @@
       <c r="E18" s="2" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G18" s="2">
+        <f t="shared" si="0"/>
+        <v>-251431614622790</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>17</v>
       </c>
@@ -10113,8 +10332,12 @@
       <c r="E19" s="2" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G19" s="2">
+        <f t="shared" si="0"/>
+        <v>1719881923523550</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>18</v>
       </c>
@@ -10130,8 +10353,12 @@
       <c r="E20" s="2" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G20" s="2">
+        <f t="shared" si="0"/>
+        <v>-228306887084200</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>19</v>
       </c>
@@ -10147,8 +10374,12 @@
       <c r="E21" s="2" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G21" s="2">
+        <f t="shared" si="0"/>
+        <v>1743370812532580</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>20</v>
       </c>
@@ -10164,8 +10395,12 @@
       <c r="E22" s="2" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G22" s="2">
+        <f t="shared" si="0"/>
+        <v>-204448101896040</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>21</v>
       </c>
@@ -10181,8 +10416,12 @@
       <c r="E23" s="2" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G23" s="2">
+        <f t="shared" si="0"/>
+        <v>1767605318917110</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>22</v>
       </c>
@@ -10199,7 +10438,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>23</v>
       </c>
@@ -10216,7 +10455,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>24</v>
       </c>
@@ -10233,7 +10472,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>25</v>
       </c>
@@ -10250,7 +10489,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>26</v>
       </c>
@@ -10267,7 +10506,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>27</v>
       </c>
@@ -10284,7 +10523,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>28</v>
       </c>
@@ -10301,7 +10540,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>29</v>
       </c>
@@ -10318,7 +10557,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>30</v>
       </c>
@@ -10913,7 +11152,7 @@
         <v>197</v>
       </c>
       <c r="F66" t="s">
-        <v>3075</v>
+        <v>3074</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
@@ -12004,7 +12243,7 @@
         <v>389</v>
       </c>
       <c r="F130" t="s">
-        <v>3075</v>
+        <v>3074</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.3">
@@ -13095,7 +13334,7 @@
         <v>581</v>
       </c>
       <c r="F194" t="s">
-        <v>3075</v>
+        <v>3074</v>
       </c>
     </row>
     <row r="195" spans="1:6" x14ac:dyDescent="0.3">
@@ -14186,7 +14425,7 @@
         <v>773</v>
       </c>
       <c r="F258" t="s">
-        <v>3075</v>
+        <v>3074</v>
       </c>
     </row>
     <row r="259" spans="1:6" x14ac:dyDescent="0.3">
@@ -15277,7 +15516,7 @@
         <v>965</v>
       </c>
       <c r="F322" t="s">
-        <v>3075</v>
+        <v>3074</v>
       </c>
     </row>
     <row r="323" spans="1:6" x14ac:dyDescent="0.3">
@@ -16368,7 +16607,7 @@
         <v>1157</v>
       </c>
       <c r="F386" t="s">
-        <v>3075</v>
+        <v>3074</v>
       </c>
     </row>
     <row r="387" spans="1:6" x14ac:dyDescent="0.3">
@@ -17459,7 +17698,7 @@
         <v>1349</v>
       </c>
       <c r="F450" t="s">
-        <v>3075</v>
+        <v>3074</v>
       </c>
     </row>
     <row r="451" spans="1:6" x14ac:dyDescent="0.3">
@@ -18550,7 +18789,7 @@
         <v>1541</v>
       </c>
       <c r="F514" t="s">
-        <v>3075</v>
+        <v>3074</v>
       </c>
     </row>
     <row r="515" spans="1:6" x14ac:dyDescent="0.3">
@@ -19641,7 +19880,7 @@
         <v>1733</v>
       </c>
       <c r="F578" t="s">
-        <v>3075</v>
+        <v>3074</v>
       </c>
     </row>
     <row r="579" spans="1:6" x14ac:dyDescent="0.3">
@@ -20732,7 +20971,7 @@
         <v>1925</v>
       </c>
       <c r="F642" t="s">
-        <v>3075</v>
+        <v>3074</v>
       </c>
     </row>
     <row r="643" spans="1:6" x14ac:dyDescent="0.3">
@@ -21823,7 +22062,7 @@
         <v>2117</v>
       </c>
       <c r="F706" t="s">
-        <v>3075</v>
+        <v>3074</v>
       </c>
     </row>
     <row r="707" spans="1:6" x14ac:dyDescent="0.3">
@@ -22914,7 +23153,7 @@
         <v>2309</v>
       </c>
       <c r="F770" t="s">
-        <v>3075</v>
+        <v>3074</v>
       </c>
     </row>
     <row r="771" spans="1:6" x14ac:dyDescent="0.3">
@@ -24005,7 +24244,7 @@
         <v>2501</v>
       </c>
       <c r="F834" t="s">
-        <v>3075</v>
+        <v>3074</v>
       </c>
     </row>
     <row r="835" spans="1:6" x14ac:dyDescent="0.3">
@@ -25096,7 +25335,7 @@
         <v>2693</v>
       </c>
       <c r="F898" t="s">
-        <v>3075</v>
+        <v>3074</v>
       </c>
     </row>
     <row r="899" spans="1:6" x14ac:dyDescent="0.3">
@@ -26187,7 +26426,7 @@
         <v>2885</v>
       </c>
       <c r="F962" t="s">
-        <v>3075</v>
+        <v>3074</v>
       </c>
     </row>
     <row r="963" spans="1:6" x14ac:dyDescent="0.3">
@@ -26458,8 +26697,8 @@
       <c r="D978" t="s">
         <v>2932</v>
       </c>
-      <c r="E978" s="2" t="s">
-        <v>2933</v>
+      <c r="E978" s="9">
+        <v>531837457726680</v>
       </c>
     </row>
     <row r="979" spans="1:5" x14ac:dyDescent="0.3">
@@ -26470,13 +26709,13 @@
         <v>-0.734375</v>
       </c>
       <c r="C979" t="s">
+        <v>2933</v>
+      </c>
+      <c r="D979" t="s">
         <v>2934</v>
       </c>
-      <c r="D979" t="s">
+      <c r="E979" s="2" t="s">
         <v>2935</v>
-      </c>
-      <c r="E979" s="2" t="s">
-        <v>2936</v>
       </c>
     </row>
     <row r="980" spans="1:5" x14ac:dyDescent="0.3">
@@ -26487,13 +26726,13 @@
         <v>-0.71875</v>
       </c>
       <c r="C980" t="s">
+        <v>2936</v>
+      </c>
+      <c r="D980" t="s">
         <v>2937</v>
       </c>
-      <c r="D980" t="s">
+      <c r="E980" s="2" t="s">
         <v>2938</v>
-      </c>
-      <c r="E980" s="2" t="s">
-        <v>2939</v>
       </c>
     </row>
     <row r="981" spans="1:5" x14ac:dyDescent="0.3">
@@ -26504,13 +26743,13 @@
         <v>-0.703125</v>
       </c>
       <c r="C981" t="s">
+        <v>2939</v>
+      </c>
+      <c r="D981" t="s">
         <v>2940</v>
       </c>
-      <c r="D981" t="s">
+      <c r="E981" s="2" t="s">
         <v>2941</v>
-      </c>
-      <c r="E981" s="2" t="s">
-        <v>2942</v>
       </c>
     </row>
     <row r="982" spans="1:5" x14ac:dyDescent="0.3">
@@ -26521,13 +26760,13 @@
         <v>-0.6875</v>
       </c>
       <c r="C982" t="s">
+        <v>2942</v>
+      </c>
+      <c r="D982" t="s">
         <v>2943</v>
       </c>
-      <c r="D982" t="s">
+      <c r="E982" s="2" t="s">
         <v>2944</v>
-      </c>
-      <c r="E982" s="2" t="s">
-        <v>2945</v>
       </c>
     </row>
     <row r="983" spans="1:5" x14ac:dyDescent="0.3">
@@ -26538,13 +26777,13 @@
         <v>-0.671875</v>
       </c>
       <c r="C983" t="s">
+        <v>2945</v>
+      </c>
+      <c r="D983" t="s">
         <v>2946</v>
       </c>
-      <c r="D983" t="s">
+      <c r="E983" s="2" t="s">
         <v>2947</v>
-      </c>
-      <c r="E983" s="2" t="s">
-        <v>2948</v>
       </c>
     </row>
     <row r="984" spans="1:5" x14ac:dyDescent="0.3">
@@ -26555,13 +26794,13 @@
         <v>-0.65625</v>
       </c>
       <c r="C984" t="s">
+        <v>2948</v>
+      </c>
+      <c r="D984" t="s">
         <v>2949</v>
       </c>
-      <c r="D984" t="s">
+      <c r="E984" s="2" t="s">
         <v>2950</v>
-      </c>
-      <c r="E984" s="2" t="s">
-        <v>2951</v>
       </c>
     </row>
     <row r="985" spans="1:5" x14ac:dyDescent="0.3">
@@ -26572,13 +26811,13 @@
         <v>-0.640625</v>
       </c>
       <c r="C985" t="s">
+        <v>2951</v>
+      </c>
+      <c r="D985" t="s">
         <v>2952</v>
       </c>
-      <c r="D985" t="s">
+      <c r="E985" s="2" t="s">
         <v>2953</v>
-      </c>
-      <c r="E985" s="2" t="s">
-        <v>2954</v>
       </c>
     </row>
     <row r="986" spans="1:5" x14ac:dyDescent="0.3">
@@ -26589,13 +26828,13 @@
         <v>-0.625</v>
       </c>
       <c r="C986" t="s">
+        <v>2954</v>
+      </c>
+      <c r="D986" t="s">
         <v>2955</v>
       </c>
-      <c r="D986" t="s">
+      <c r="E986" s="2" t="s">
         <v>2956</v>
-      </c>
-      <c r="E986" s="2" t="s">
-        <v>2957</v>
       </c>
     </row>
     <row r="987" spans="1:5" x14ac:dyDescent="0.3">
@@ -26606,13 +26845,13 @@
         <v>-0.609375</v>
       </c>
       <c r="C987" t="s">
+        <v>2957</v>
+      </c>
+      <c r="D987" t="s">
         <v>2958</v>
       </c>
-      <c r="D987" t="s">
+      <c r="E987" s="2" t="s">
         <v>2959</v>
-      </c>
-      <c r="E987" s="2" t="s">
-        <v>2960</v>
       </c>
     </row>
     <row r="988" spans="1:5" x14ac:dyDescent="0.3">
@@ -26623,13 +26862,13 @@
         <v>-0.59375</v>
       </c>
       <c r="C988" t="s">
+        <v>2960</v>
+      </c>
+      <c r="D988" t="s">
         <v>2961</v>
       </c>
-      <c r="D988" t="s">
+      <c r="E988" s="2" t="s">
         <v>2962</v>
-      </c>
-      <c r="E988" s="2" t="s">
-        <v>2963</v>
       </c>
     </row>
     <row r="989" spans="1:5" x14ac:dyDescent="0.3">
@@ -26640,13 +26879,13 @@
         <v>-0.578125</v>
       </c>
       <c r="C989" t="s">
+        <v>2963</v>
+      </c>
+      <c r="D989" t="s">
         <v>2964</v>
       </c>
-      <c r="D989" t="s">
+      <c r="E989" s="2" t="s">
         <v>2965</v>
-      </c>
-      <c r="E989" s="2" t="s">
-        <v>2966</v>
       </c>
     </row>
     <row r="990" spans="1:5" x14ac:dyDescent="0.3">
@@ -26657,13 +26896,13 @@
         <v>-0.5625</v>
       </c>
       <c r="C990" t="s">
+        <v>2966</v>
+      </c>
+      <c r="D990" t="s">
         <v>2967</v>
       </c>
-      <c r="D990" t="s">
+      <c r="E990" s="2" t="s">
         <v>2968</v>
-      </c>
-      <c r="E990" s="2" t="s">
-        <v>2969</v>
       </c>
     </row>
     <row r="991" spans="1:5" x14ac:dyDescent="0.3">
@@ -26674,13 +26913,13 @@
         <v>-0.546875</v>
       </c>
       <c r="C991" t="s">
+        <v>2969</v>
+      </c>
+      <c r="D991" t="s">
         <v>2970</v>
       </c>
-      <c r="D991" t="s">
+      <c r="E991" s="2" t="s">
         <v>2971</v>
-      </c>
-      <c r="E991" s="2" t="s">
-        <v>2972</v>
       </c>
     </row>
     <row r="992" spans="1:5" x14ac:dyDescent="0.3">
@@ -26691,13 +26930,13 @@
         <v>-0.53125</v>
       </c>
       <c r="C992" t="s">
+        <v>2972</v>
+      </c>
+      <c r="D992" t="s">
         <v>2973</v>
       </c>
-      <c r="D992" t="s">
+      <c r="E992" s="2" t="s">
         <v>2974</v>
-      </c>
-      <c r="E992" s="2" t="s">
-        <v>2975</v>
       </c>
     </row>
     <row r="993" spans="1:5" x14ac:dyDescent="0.3">
@@ -26708,13 +26947,13 @@
         <v>-0.515625</v>
       </c>
       <c r="C993" t="s">
+        <v>2975</v>
+      </c>
+      <c r="D993" t="s">
         <v>2976</v>
       </c>
-      <c r="D993" t="s">
+      <c r="E993" s="2" t="s">
         <v>2977</v>
-      </c>
-      <c r="E993" s="2" t="s">
-        <v>2978</v>
       </c>
     </row>
     <row r="994" spans="1:5" x14ac:dyDescent="0.3">
@@ -26725,13 +26964,13 @@
         <v>-0.5</v>
       </c>
       <c r="C994" t="s">
+        <v>2978</v>
+      </c>
+      <c r="D994" t="s">
         <v>2979</v>
       </c>
-      <c r="D994" t="s">
+      <c r="E994" s="2" t="s">
         <v>2980</v>
-      </c>
-      <c r="E994" s="2" t="s">
-        <v>2981</v>
       </c>
     </row>
     <row r="995" spans="1:5" x14ac:dyDescent="0.3">
@@ -26742,13 +26981,13 @@
         <v>-0.484375</v>
       </c>
       <c r="C995" t="s">
+        <v>2981</v>
+      </c>
+      <c r="D995" t="s">
         <v>2982</v>
       </c>
-      <c r="D995" t="s">
+      <c r="E995" s="2" t="s">
         <v>2983</v>
-      </c>
-      <c r="E995" s="2" t="s">
-        <v>2984</v>
       </c>
     </row>
     <row r="996" spans="1:5" x14ac:dyDescent="0.3">
@@ -26759,13 +26998,13 @@
         <v>-0.46875</v>
       </c>
       <c r="C996" t="s">
+        <v>2984</v>
+      </c>
+      <c r="D996" t="s">
         <v>2985</v>
       </c>
-      <c r="D996" t="s">
+      <c r="E996" s="2" t="s">
         <v>2986</v>
-      </c>
-      <c r="E996" s="2" t="s">
-        <v>2987</v>
       </c>
     </row>
     <row r="997" spans="1:5" x14ac:dyDescent="0.3">
@@ -26776,13 +27015,13 @@
         <v>-0.453125</v>
       </c>
       <c r="C997" t="s">
+        <v>2987</v>
+      </c>
+      <c r="D997" t="s">
         <v>2988</v>
       </c>
-      <c r="D997" t="s">
+      <c r="E997" s="2" t="s">
         <v>2989</v>
-      </c>
-      <c r="E997" s="2" t="s">
-        <v>2990</v>
       </c>
     </row>
     <row r="998" spans="1:5" x14ac:dyDescent="0.3">
@@ -26793,13 +27032,13 @@
         <v>-0.4375</v>
       </c>
       <c r="C998" t="s">
+        <v>2990</v>
+      </c>
+      <c r="D998" t="s">
         <v>2991</v>
       </c>
-      <c r="D998" t="s">
+      <c r="E998" s="2" t="s">
         <v>2992</v>
-      </c>
-      <c r="E998" s="2" t="s">
-        <v>2993</v>
       </c>
     </row>
     <row r="999" spans="1:5" x14ac:dyDescent="0.3">
@@ -26810,13 +27049,13 @@
         <v>-0.421875</v>
       </c>
       <c r="C999" t="s">
+        <v>2993</v>
+      </c>
+      <c r="D999" t="s">
         <v>2994</v>
       </c>
-      <c r="D999" t="s">
+      <c r="E999" s="2" t="s">
         <v>2995</v>
-      </c>
-      <c r="E999" s="2" t="s">
-        <v>2996</v>
       </c>
     </row>
     <row r="1000" spans="1:5" x14ac:dyDescent="0.3">
@@ -26827,13 +27066,13 @@
         <v>-0.40625</v>
       </c>
       <c r="C1000" t="s">
+        <v>2996</v>
+      </c>
+      <c r="D1000" t="s">
         <v>2997</v>
       </c>
-      <c r="D1000" t="s">
+      <c r="E1000" s="2" t="s">
         <v>2998</v>
-      </c>
-      <c r="E1000" s="2" t="s">
-        <v>2999</v>
       </c>
     </row>
     <row r="1001" spans="1:5" x14ac:dyDescent="0.3">
@@ -26844,13 +27083,13 @@
         <v>-0.390625</v>
       </c>
       <c r="C1001" t="s">
+        <v>2999</v>
+      </c>
+      <c r="D1001" t="s">
         <v>3000</v>
       </c>
-      <c r="D1001" t="s">
+      <c r="E1001" s="2" t="s">
         <v>3001</v>
-      </c>
-      <c r="E1001" s="2" t="s">
-        <v>3002</v>
       </c>
     </row>
     <row r="1002" spans="1:5" x14ac:dyDescent="0.3">
@@ -26861,13 +27100,13 @@
         <v>-0.375</v>
       </c>
       <c r="C1002" t="s">
+        <v>3002</v>
+      </c>
+      <c r="D1002" t="s">
         <v>3003</v>
       </c>
-      <c r="D1002" t="s">
+      <c r="E1002" s="2" t="s">
         <v>3004</v>
-      </c>
-      <c r="E1002" s="2" t="s">
-        <v>3005</v>
       </c>
     </row>
     <row r="1003" spans="1:5" x14ac:dyDescent="0.3">
@@ -26878,13 +27117,13 @@
         <v>-0.359375</v>
       </c>
       <c r="C1003" t="s">
+        <v>3005</v>
+      </c>
+      <c r="D1003" t="s">
         <v>3006</v>
       </c>
-      <c r="D1003" t="s">
+      <c r="E1003" s="2" t="s">
         <v>3007</v>
-      </c>
-      <c r="E1003" s="2" t="s">
-        <v>3008</v>
       </c>
     </row>
     <row r="1004" spans="1:5" x14ac:dyDescent="0.3">
@@ -26895,13 +27134,13 @@
         <v>-0.34375</v>
       </c>
       <c r="C1004" t="s">
+        <v>3008</v>
+      </c>
+      <c r="D1004" t="s">
         <v>3009</v>
       </c>
-      <c r="D1004" t="s">
+      <c r="E1004" s="2" t="s">
         <v>3010</v>
-      </c>
-      <c r="E1004" s="2" t="s">
-        <v>3011</v>
       </c>
     </row>
     <row r="1005" spans="1:5" x14ac:dyDescent="0.3">
@@ -26912,13 +27151,13 @@
         <v>-0.328125</v>
       </c>
       <c r="C1005" t="s">
+        <v>3011</v>
+      </c>
+      <c r="D1005" t="s">
         <v>3012</v>
       </c>
-      <c r="D1005" t="s">
+      <c r="E1005" s="2" t="s">
         <v>3013</v>
-      </c>
-      <c r="E1005" s="2" t="s">
-        <v>3014</v>
       </c>
     </row>
     <row r="1006" spans="1:5" x14ac:dyDescent="0.3">
@@ -26929,13 +27168,13 @@
         <v>-0.3125</v>
       </c>
       <c r="C1006" t="s">
+        <v>3014</v>
+      </c>
+      <c r="D1006" t="s">
         <v>3015</v>
       </c>
-      <c r="D1006" t="s">
+      <c r="E1006" s="2" t="s">
         <v>3016</v>
-      </c>
-      <c r="E1006" s="2" t="s">
-        <v>3017</v>
       </c>
     </row>
     <row r="1007" spans="1:5" x14ac:dyDescent="0.3">
@@ -26946,13 +27185,13 @@
         <v>-0.296875</v>
       </c>
       <c r="C1007" t="s">
+        <v>3017</v>
+      </c>
+      <c r="D1007" t="s">
         <v>3018</v>
       </c>
-      <c r="D1007" t="s">
+      <c r="E1007" s="2" t="s">
         <v>3019</v>
-      </c>
-      <c r="E1007" s="2" t="s">
-        <v>3020</v>
       </c>
     </row>
     <row r="1008" spans="1:5" x14ac:dyDescent="0.3">
@@ -26963,13 +27202,13 @@
         <v>-0.28125</v>
       </c>
       <c r="C1008" t="s">
+        <v>3020</v>
+      </c>
+      <c r="D1008" t="s">
         <v>3021</v>
       </c>
-      <c r="D1008" t="s">
+      <c r="E1008" s="2" t="s">
         <v>3022</v>
-      </c>
-      <c r="E1008" s="2" t="s">
-        <v>3023</v>
       </c>
     </row>
     <row r="1009" spans="1:5" x14ac:dyDescent="0.3">
@@ -26980,13 +27219,13 @@
         <v>-0.265625</v>
       </c>
       <c r="C1009" t="s">
+        <v>3023</v>
+      </c>
+      <c r="D1009" t="s">
         <v>3024</v>
       </c>
-      <c r="D1009" t="s">
+      <c r="E1009" s="2" t="s">
         <v>3025</v>
-      </c>
-      <c r="E1009" s="2" t="s">
-        <v>3026</v>
       </c>
     </row>
     <row r="1010" spans="1:5" x14ac:dyDescent="0.3">
@@ -26997,13 +27236,13 @@
         <v>-0.25</v>
       </c>
       <c r="C1010" t="s">
+        <v>3026</v>
+      </c>
+      <c r="D1010" t="s">
         <v>3027</v>
       </c>
-      <c r="D1010" t="s">
+      <c r="E1010" s="2" t="s">
         <v>3028</v>
-      </c>
-      <c r="E1010" s="2" t="s">
-        <v>3029</v>
       </c>
     </row>
     <row r="1011" spans="1:5" x14ac:dyDescent="0.3">
@@ -27014,13 +27253,13 @@
         <v>-0.234375</v>
       </c>
       <c r="C1011" t="s">
+        <v>3029</v>
+      </c>
+      <c r="D1011" t="s">
         <v>3030</v>
       </c>
-      <c r="D1011" t="s">
+      <c r="E1011" s="2" t="s">
         <v>3031</v>
-      </c>
-      <c r="E1011" s="2" t="s">
-        <v>3032</v>
       </c>
     </row>
     <row r="1012" spans="1:5" x14ac:dyDescent="0.3">
@@ -27031,13 +27270,13 @@
         <v>-0.21875</v>
       </c>
       <c r="C1012" t="s">
+        <v>3032</v>
+      </c>
+      <c r="D1012" t="s">
         <v>3033</v>
       </c>
-      <c r="D1012" t="s">
+      <c r="E1012" s="2" t="s">
         <v>3034</v>
-      </c>
-      <c r="E1012" s="2" t="s">
-        <v>3035</v>
       </c>
     </row>
     <row r="1013" spans="1:5" x14ac:dyDescent="0.3">
@@ -27048,13 +27287,13 @@
         <v>-0.203125</v>
       </c>
       <c r="C1013" t="s">
+        <v>3035</v>
+      </c>
+      <c r="D1013" t="s">
         <v>3036</v>
       </c>
-      <c r="D1013" t="s">
+      <c r="E1013" s="2" t="s">
         <v>3037</v>
-      </c>
-      <c r="E1013" s="2" t="s">
-        <v>3038</v>
       </c>
     </row>
     <row r="1014" spans="1:5" x14ac:dyDescent="0.3">
@@ -27065,13 +27304,13 @@
         <v>-0.1875</v>
       </c>
       <c r="C1014" t="s">
+        <v>3038</v>
+      </c>
+      <c r="D1014" t="s">
         <v>3039</v>
       </c>
-      <c r="D1014" t="s">
+      <c r="E1014" s="2" t="s">
         <v>3040</v>
-      </c>
-      <c r="E1014" s="2" t="s">
-        <v>3041</v>
       </c>
     </row>
     <row r="1015" spans="1:5" x14ac:dyDescent="0.3">
@@ -27082,13 +27321,13 @@
         <v>-0.171875</v>
       </c>
       <c r="C1015" t="s">
+        <v>3041</v>
+      </c>
+      <c r="D1015" t="s">
         <v>3042</v>
       </c>
-      <c r="D1015" t="s">
+      <c r="E1015" s="2" t="s">
         <v>3043</v>
-      </c>
-      <c r="E1015" s="2" t="s">
-        <v>3044</v>
       </c>
     </row>
     <row r="1016" spans="1:5" x14ac:dyDescent="0.3">
@@ -27099,13 +27338,13 @@
         <v>-0.15625</v>
       </c>
       <c r="C1016" t="s">
+        <v>3044</v>
+      </c>
+      <c r="D1016" t="s">
         <v>3045</v>
       </c>
-      <c r="D1016" t="s">
+      <c r="E1016" s="2" t="s">
         <v>3046</v>
-      </c>
-      <c r="E1016" s="2" t="s">
-        <v>3047</v>
       </c>
     </row>
     <row r="1017" spans="1:5" x14ac:dyDescent="0.3">
@@ -27116,13 +27355,13 @@
         <v>-0.140625</v>
       </c>
       <c r="C1017" t="s">
+        <v>3047</v>
+      </c>
+      <c r="D1017" t="s">
         <v>3048</v>
       </c>
-      <c r="D1017" t="s">
+      <c r="E1017" s="2" t="s">
         <v>3049</v>
-      </c>
-      <c r="E1017" s="2" t="s">
-        <v>3050</v>
       </c>
     </row>
     <row r="1018" spans="1:5" x14ac:dyDescent="0.3">
@@ -27133,13 +27372,13 @@
         <v>-0.125</v>
       </c>
       <c r="C1018" t="s">
+        <v>3050</v>
+      </c>
+      <c r="D1018" t="s">
         <v>3051</v>
       </c>
-      <c r="D1018" t="s">
+      <c r="E1018" s="2" t="s">
         <v>3052</v>
-      </c>
-      <c r="E1018" s="2" t="s">
-        <v>3053</v>
       </c>
     </row>
     <row r="1019" spans="1:5" x14ac:dyDescent="0.3">
@@ -27150,13 +27389,13 @@
         <v>-0.109375</v>
       </c>
       <c r="C1019" t="s">
+        <v>3053</v>
+      </c>
+      <c r="D1019" t="s">
         <v>3054</v>
       </c>
-      <c r="D1019" t="s">
+      <c r="E1019" s="2" t="s">
         <v>3055</v>
-      </c>
-      <c r="E1019" s="2" t="s">
-        <v>3056</v>
       </c>
     </row>
     <row r="1020" spans="1:5" x14ac:dyDescent="0.3">
@@ -27167,13 +27406,13 @@
         <v>-9.375E-2</v>
       </c>
       <c r="C1020" t="s">
+        <v>3056</v>
+      </c>
+      <c r="D1020" t="s">
         <v>3057</v>
       </c>
-      <c r="D1020" t="s">
+      <c r="E1020" s="2" t="s">
         <v>3058</v>
-      </c>
-      <c r="E1020" s="2" t="s">
-        <v>3059</v>
       </c>
     </row>
     <row r="1021" spans="1:5" x14ac:dyDescent="0.3">
@@ -27184,13 +27423,13 @@
         <v>-7.8125E-2</v>
       </c>
       <c r="C1021" t="s">
+        <v>3059</v>
+      </c>
+      <c r="D1021" t="s">
         <v>3060</v>
       </c>
-      <c r="D1021" t="s">
+      <c r="E1021" s="2" t="s">
         <v>3061</v>
-      </c>
-      <c r="E1021" s="2" t="s">
-        <v>3062</v>
       </c>
     </row>
     <row r="1022" spans="1:5" x14ac:dyDescent="0.3">
@@ -27201,13 +27440,13 @@
         <v>-6.25E-2</v>
       </c>
       <c r="C1022" t="s">
+        <v>3062</v>
+      </c>
+      <c r="D1022" t="s">
         <v>3063</v>
       </c>
-      <c r="D1022" t="s">
+      <c r="E1022" s="2" t="s">
         <v>3064</v>
-      </c>
-      <c r="E1022" s="2" t="s">
-        <v>3065</v>
       </c>
     </row>
     <row r="1023" spans="1:5" x14ac:dyDescent="0.3">
@@ -27218,13 +27457,13 @@
         <v>-4.6875E-2</v>
       </c>
       <c r="C1023" t="s">
+        <v>3065</v>
+      </c>
+      <c r="D1023" t="s">
         <v>3066</v>
       </c>
-      <c r="D1023" t="s">
+      <c r="E1023" s="2" t="s">
         <v>3067</v>
-      </c>
-      <c r="E1023" s="2" t="s">
-        <v>3068</v>
       </c>
     </row>
     <row r="1024" spans="1:5" x14ac:dyDescent="0.3">
@@ -27235,13 +27474,13 @@
         <v>-3.125E-2</v>
       </c>
       <c r="C1024" t="s">
+        <v>3068</v>
+      </c>
+      <c r="D1024" t="s">
         <v>3069</v>
       </c>
-      <c r="D1024" t="s">
+      <c r="E1024" s="2" t="s">
         <v>3070</v>
-      </c>
-      <c r="E1024" s="2" t="s">
-        <v>3071</v>
       </c>
     </row>
     <row r="1025" spans="1:6" x14ac:dyDescent="0.3">
@@ -27252,43 +27491,43 @@
         <v>-1.5625E-2</v>
       </c>
       <c r="C1025" t="s">
+        <v>3071</v>
+      </c>
+      <c r="D1025" t="s">
         <v>3072</v>
       </c>
-      <c r="D1025" t="s">
+      <c r="E1025" s="2" t="s">
         <v>3073</v>
       </c>
-      <c r="E1025" s="2" t="s">
-        <v>3074</v>
-      </c>
     </row>
     <row r="1028" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1028" s="8" t="s">
-        <v>3090</v>
-      </c>
-      <c r="B1028" s="9"/>
-      <c r="C1028" s="9"/>
-      <c r="D1028" s="9"/>
-      <c r="E1028" s="9"/>
-      <c r="F1028" s="10"/>
+      <c r="A1028" s="10" t="s">
+        <v>3089</v>
+      </c>
+      <c r="B1028" s="11"/>
+      <c r="C1028" s="11"/>
+      <c r="D1028" s="11"/>
+      <c r="E1028" s="11"/>
+      <c r="F1028" s="12"/>
     </row>
     <row r="1029" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1029" t="s">
+        <v>3075</v>
+      </c>
+      <c r="B1029" t="s">
         <v>3076</v>
       </c>
-      <c r="B1029" t="s">
+      <c r="C1029" t="s">
         <v>3077</v>
       </c>
-      <c r="C1029" t="s">
+      <c r="D1029" t="s">
         <v>3078</v>
       </c>
-      <c r="D1029" t="s">
+      <c r="E1029" t="s">
+        <v>3080</v>
+      </c>
+      <c r="F1029" t="s">
         <v>3079</v>
-      </c>
-      <c r="E1029" t="s">
-        <v>3081</v>
-      </c>
-      <c r="F1029" t="s">
-        <v>3080</v>
       </c>
     </row>
     <row r="1030" spans="1:6" x14ac:dyDescent="0.3">
@@ -27315,40 +27554,40 @@
       </c>
     </row>
     <row r="1041" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1041" s="8" t="s">
-        <v>3089</v>
-      </c>
-      <c r="B1041" s="9"/>
-      <c r="C1041" s="9"/>
-      <c r="D1041" s="9"/>
-      <c r="E1041" s="9"/>
-      <c r="F1041" s="9"/>
-      <c r="G1041" s="10"/>
+      <c r="A1041" s="10" t="s">
+        <v>3088</v>
+      </c>
+      <c r="B1041" s="11"/>
+      <c r="C1041" s="11"/>
+      <c r="D1041" s="11"/>
+      <c r="E1041" s="11"/>
+      <c r="F1041" s="11"/>
+      <c r="G1041" s="12"/>
     </row>
     <row r="1042" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1042" t="s">
+        <v>3081</v>
+      </c>
+      <c r="B1042" t="s">
         <v>3082</v>
       </c>
-      <c r="B1042" t="s">
+      <c r="C1042" t="s">
         <v>3083</v>
       </c>
-      <c r="C1042" t="s">
+      <c r="D1042" t="s">
         <v>3084</v>
       </c>
-      <c r="D1042" t="s">
+      <c r="E1042" t="s">
         <v>3085</v>
       </c>
-      <c r="E1042" t="s">
+      <c r="F1042" t="s">
         <v>3086</v>
       </c>
-      <c r="F1042" t="s">
+      <c r="G1042" t="s">
         <v>3087</v>
       </c>
-      <c r="G1042" t="s">
-        <v>3088</v>
-      </c>
       <c r="H1042" t="s">
-        <v>3091</v>
+        <v>3090</v>
       </c>
     </row>
     <row r="1043" spans="1:8" x14ac:dyDescent="0.3">
@@ -27413,7 +27652,7 @@
         <v>1.2207031250005551E-4</v>
       </c>
       <c r="H1044" s="6">
-        <f t="shared" ref="H1044:H1046" si="0">(F1044-C1044)/C1044</f>
+        <f t="shared" ref="H1044:H1046" si="1">(F1044-C1044)/C1044</f>
         <v>1.2207031250005551E-4</v>
       </c>
     </row>
@@ -27446,7 +27685,7 @@
         <v>2.3282020331068849E-10</v>
       </c>
       <c r="H1045" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2.3282020331068849E-10</v>
       </c>
     </row>
@@ -27455,7 +27694,7 @@
         <v>20</v>
       </c>
       <c r="B1046">
-        <f t="shared" ref="B1046:B1047" si="1">2^A1046</f>
+        <f t="shared" ref="B1046" si="2">2^A1046</f>
         <v>1048576</v>
       </c>
       <c r="C1046">
@@ -27463,23 +27702,23 @@
         <v>3.3546262790251185E-4</v>
       </c>
       <c r="D1046">
-        <f t="shared" ref="D1046:D1047" si="2">C1046*B1046</f>
+        <f t="shared" ref="D1046" si="3">C1046*B1046</f>
         <v>351.75806051550427</v>
       </c>
       <c r="E1046" s="7">
-        <f t="shared" ref="E1046:E1047" si="3">ROUND(D1046,0)</f>
+        <f t="shared" ref="E1046" si="4">ROUND(D1046,0)</f>
         <v>352</v>
       </c>
       <c r="F1046">
-        <f t="shared" ref="F1046:F1047" si="4">E1046/B1046</f>
+        <f t="shared" ref="F1046" si="5">E1046/B1046</f>
         <v>3.35693359375E-4</v>
       </c>
       <c r="G1046" s="4">
-        <f t="shared" ref="G1046:G1047" si="5">(F1046-C1046)/C1046</f>
+        <f t="shared" ref="G1046" si="6">(F1046-C1046)/C1046</f>
         <v>6.8780082577543991E-4</v>
       </c>
       <c r="H1046" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6.8780082577543991E-4</v>
       </c>
     </row>
@@ -27493,10 +27732,278 @@
         <v>1.5625E-2</v>
       </c>
     </row>
+    <row r="1050" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1050" s="10" t="s">
+        <v>3124</v>
+      </c>
+      <c r="B1050" s="11"/>
+      <c r="C1050" s="11"/>
+      <c r="D1050" s="11"/>
+      <c r="E1050" s="11"/>
+      <c r="F1050" s="11"/>
+      <c r="G1050" s="12"/>
+    </row>
+    <row r="1051" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="C1051" t="s">
+        <v>3116</v>
+      </c>
+      <c r="D1051" t="s">
+        <v>3117</v>
+      </c>
+    </row>
+    <row r="1052" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="C1052">
+        <v>976</v>
+      </c>
+      <c r="D1052">
+        <v>6</v>
+      </c>
+      <c r="F1052" t="s">
+        <v>3118</v>
+      </c>
+    </row>
+    <row r="1053" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1053" t="s">
+        <v>3121</v>
+      </c>
+    </row>
+    <row r="1054" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1054" t="s">
+        <v>3092</v>
+      </c>
+      <c r="B1054" t="s">
+        <v>3101</v>
+      </c>
+      <c r="C1054">
+        <f>D1052*E1054</f>
+        <v>4098</v>
+      </c>
+      <c r="E1054">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="1055" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1055" t="s">
+        <v>3093</v>
+      </c>
+      <c r="B1055" t="s">
+        <v>3102</v>
+      </c>
+      <c r="C1055">
+        <f>C1054+G1055</f>
+        <v>47794</v>
+      </c>
+      <c r="E1055" t="s">
+        <v>3107</v>
+      </c>
+      <c r="F1055" t="s">
+        <v>3108</v>
+      </c>
+      <c r="G1055">
+        <f>2731*16</f>
+        <v>43696</v>
+      </c>
+      <c r="H1055">
+        <v>2731</v>
+      </c>
+    </row>
+    <row r="1056" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1056" t="s">
+        <v>3094</v>
+      </c>
+      <c r="B1056" t="s">
+        <v>3103</v>
+      </c>
+      <c r="C1056">
+        <f>C1055*D1052</f>
+        <v>286764</v>
+      </c>
+      <c r="E1056">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1057" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1057" t="s">
+        <v>3095</v>
+      </c>
+      <c r="B1057" t="s">
+        <v>3104</v>
+      </c>
+      <c r="C1057">
+        <f>C1056+G1057</f>
+        <v>2383916</v>
+      </c>
+      <c r="E1057" t="s">
+        <v>3110</v>
+      </c>
+      <c r="F1057" t="s">
+        <v>3109</v>
+      </c>
+      <c r="G1057">
+        <f>2^21</f>
+        <v>2097152</v>
+      </c>
+    </row>
+    <row r="1058" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1058" t="s">
+        <v>3096</v>
+      </c>
+      <c r="B1058" t="s">
+        <v>3103</v>
+      </c>
+      <c r="C1058">
+        <f>C1057*D1052</f>
+        <v>14303496</v>
+      </c>
+      <c r="E1058">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1059" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1059" t="s">
+        <v>3097</v>
+      </c>
+      <c r="B1059" t="s">
+        <v>3105</v>
+      </c>
+      <c r="C1059">
+        <f>C1058+G1059</f>
+        <v>81412360</v>
+      </c>
+      <c r="E1059" t="s">
+        <v>3111</v>
+      </c>
+      <c r="F1059" t="s">
+        <v>3112</v>
+      </c>
+      <c r="G1059">
+        <f>2^26</f>
+        <v>67108864</v>
+      </c>
+    </row>
+    <row r="1060" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1060" t="s">
+        <v>3098</v>
+      </c>
+      <c r="B1060" t="s">
+        <v>3103</v>
+      </c>
+      <c r="C1060">
+        <f>C1059*D1052</f>
+        <v>488474160</v>
+      </c>
+      <c r="E1060">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1061" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1061" t="s">
+        <v>3099</v>
+      </c>
+      <c r="B1061" t="s">
+        <v>3105</v>
+      </c>
+      <c r="C1061">
+        <f>C1060+G1061</f>
+        <v>1562215984</v>
+      </c>
+      <c r="E1061" t="s">
+        <v>3113</v>
+      </c>
+      <c r="F1061" t="s">
+        <v>3114</v>
+      </c>
+      <c r="G1061">
+        <f>2^30</f>
+        <v>1073741824</v>
+      </c>
+    </row>
+    <row r="1062" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1062" t="s">
+        <v>3100</v>
+      </c>
+      <c r="B1062" t="s">
+        <v>3106</v>
+      </c>
+      <c r="C1062" s="2">
+        <f>C1061*495312</f>
+        <v>773784323467008</v>
+      </c>
+      <c r="F1062" t="s">
+        <v>3115</v>
+      </c>
+      <c r="G1062" s="2">
+        <f>495312*2^30</f>
+        <v>531837210329088</v>
+      </c>
+    </row>
+    <row r="1063" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F1063" t="s">
+        <v>3119</v>
+      </c>
+      <c r="G1063" s="2">
+        <v>531837457726680</v>
+      </c>
+    </row>
+    <row r="1064" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1064" t="s">
+        <v>3120</v>
+      </c>
+      <c r="C1064" s="2">
+        <f>C1062-E978</f>
+        <v>241946865740328</v>
+      </c>
+    </row>
+    <row r="1065" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1065" t="s">
+        <v>3079</v>
+      </c>
+      <c r="C1065">
+        <f>(C1062-E984)/E984</f>
+        <v>0.32472550354327395</v>
+      </c>
+    </row>
+    <row r="1066" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D1066" s="2"/>
+    </row>
+    <row r="1068" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C1068" s="9">
+        <v>531837457726680</v>
+      </c>
+    </row>
+    <row r="1072" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1072">
+        <v>-0.75</v>
+      </c>
+      <c r="B1072">
+        <f>EXP(A1072)</f>
+        <v>0.47236655274101469</v>
+      </c>
+      <c r="D1072" t="s">
+        <v>3122</v>
+      </c>
+    </row>
+    <row r="1073" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1073">
+        <v>-0.65625</v>
+      </c>
+      <c r="B1073">
+        <f>EXP(A1073)</f>
+        <v>0.51879316565388933</v>
+      </c>
+      <c r="D1073" t="s">
+        <v>3123</v>
+      </c>
+      <c r="E1073">
+        <f>B1072+B1072*(A1073-A1072)+B1072/2*(A1073-A1072)^2+B1072/6*(A1073-A1072)^3+B1072/24*(A1073-A1072)^4</f>
+        <v>0.5187931366952474</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1041:G1041"/>
     <mergeCell ref="A1028:F1028"/>
+    <mergeCell ref="A1050:G1050"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
2025.11.21 fix the softmax function
</commit_message>
<xml_diff>
--- a/HW5/Softmax_table.xlsx
+++ b/HW5/Softmax_table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c1d8b65b6adf7979/桌面/Github File/IC_Design_Laboratory/HW5/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="503" documentId="11_1B85D0BDD370594FA3B82111595ED87656CB84C1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8E8EEAA7-F43D-4855-879D-B5987E5E595E}"/>
+  <xr:revisionPtr revIDLastSave="518" documentId="11_1B85D0BDD370594FA3B82111595ED87656CB84C1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6B320B9E-173E-4FED-B3E4-F279406CC2FE}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3157" uniqueCount="3137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3168" uniqueCount="3137">
   <si>
     <t>Fixed-point Input (4Q6)</t>
   </si>
@@ -9666,11 +9666,11 @@
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -9978,7 +9978,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H1087"/>
+  <dimension ref="A1:H1097"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="25.19921875" bestFit="1" customWidth="1"/>
@@ -27557,14 +27557,14 @@
       </c>
     </row>
     <row r="1028" spans="1:6">
-      <c r="A1028" s="10" t="s">
+      <c r="A1028" s="12" t="s">
         <v>3089</v>
       </c>
-      <c r="B1028" s="11"/>
-      <c r="C1028" s="11"/>
-      <c r="D1028" s="11"/>
-      <c r="E1028" s="11"/>
-      <c r="F1028" s="12"/>
+      <c r="B1028" s="13"/>
+      <c r="C1028" s="13"/>
+      <c r="D1028" s="13"/>
+      <c r="E1028" s="13"/>
+      <c r="F1028" s="14"/>
     </row>
     <row r="1029" spans="1:6">
       <c r="A1029" t="s">
@@ -27610,15 +27610,15 @@
       </c>
     </row>
     <row r="1041" spans="1:8">
-      <c r="A1041" s="10" t="s">
+      <c r="A1041" s="12" t="s">
         <v>3088</v>
       </c>
-      <c r="B1041" s="11"/>
-      <c r="C1041" s="11"/>
-      <c r="D1041" s="11"/>
-      <c r="E1041" s="11"/>
-      <c r="F1041" s="11"/>
-      <c r="G1041" s="12"/>
+      <c r="B1041" s="13"/>
+      <c r="C1041" s="13"/>
+      <c r="D1041" s="13"/>
+      <c r="E1041" s="13"/>
+      <c r="F1041" s="13"/>
+      <c r="G1041" s="14"/>
     </row>
     <row r="1042" spans="1:8">
       <c r="A1042" t="s">
@@ -27789,15 +27789,15 @@
       </c>
     </row>
     <row r="1050" spans="1:8">
-      <c r="A1050" s="10" t="s">
+      <c r="A1050" s="12" t="s">
         <v>3124</v>
       </c>
-      <c r="B1050" s="11"/>
-      <c r="C1050" s="11"/>
-      <c r="D1050" s="11"/>
-      <c r="E1050" s="11"/>
-      <c r="F1050" s="11"/>
-      <c r="G1050" s="12"/>
+      <c r="B1050" s="13"/>
+      <c r="C1050" s="13"/>
+      <c r="D1050" s="13"/>
+      <c r="E1050" s="13"/>
+      <c r="F1050" s="13"/>
+      <c r="G1050" s="14"/>
     </row>
     <row r="1051" spans="1:8">
       <c r="C1051" t="s">
@@ -28056,7 +28056,7 @@
       </c>
     </row>
     <row r="1078" spans="1:5" ht="15">
-      <c r="A1078" s="13" t="s">
+      <c r="A1078" s="10" t="s">
         <v>3125</v>
       </c>
     </row>
@@ -28081,7 +28081,7 @@
       <c r="C1080">
         <v>969774</v>
       </c>
-      <c r="D1080" s="14">
+      <c r="D1080" s="11">
         <f>ROUNDDOWN(C1080/2^16,0)</f>
         <v>14</v>
       </c>
@@ -28100,7 +28100,7 @@
       <c r="C1081">
         <v>59855117</v>
       </c>
-      <c r="D1081" s="14">
+      <c r="D1081" s="11">
         <f>ROUNDDOWN(C1081/2^16,0)</f>
         <v>913</v>
       </c>
@@ -28131,12 +28131,15 @@
         <v>3136</v>
       </c>
       <c r="C1083">
+        <f>ROUNDDOWN(C1082/C1086,0)</f>
         <v>1</v>
       </c>
       <c r="D1083">
+        <f>ROUNDDOWN(D1082/D1086,0)</f>
         <v>0</v>
       </c>
       <c r="E1083">
+        <f>ROUNDDOWN(E1082/E1086,0)</f>
         <v>1</v>
       </c>
     </row>
@@ -28148,9 +28151,122 @@
         <f>1/2^6</f>
         <v>1.5625E-2</v>
       </c>
+      <c r="D1086">
+        <f t="shared" ref="D1086:E1086" si="7">1/2^6</f>
+        <v>1.5625E-2</v>
+      </c>
+      <c r="E1086">
+        <f t="shared" si="7"/>
+        <v>1.5625E-2</v>
+      </c>
     </row>
     <row r="1087" spans="1:5">
       <c r="B1087" t="s">
+        <v>3135</v>
+      </c>
+    </row>
+    <row r="1089" spans="1:5">
+      <c r="C1089" t="s">
+        <v>3132</v>
+      </c>
+      <c r="D1089" t="s">
+        <v>3131</v>
+      </c>
+      <c r="E1089" t="s">
+        <v>3134</v>
+      </c>
+    </row>
+    <row r="1090" spans="1:5">
+      <c r="A1090" t="s">
+        <v>3127</v>
+      </c>
+      <c r="B1090" t="s">
+        <v>3129</v>
+      </c>
+      <c r="C1090">
+        <v>1284742</v>
+      </c>
+      <c r="D1090" s="11">
+        <f>ROUNDDOWN(C1090/2^16,0)</f>
+        <v>19</v>
+      </c>
+      <c r="E1090">
+        <f>ROUNDDOWN(C1090/2^14,0)</f>
+        <v>78</v>
+      </c>
+    </row>
+    <row r="1091" spans="1:5">
+      <c r="A1091" t="s">
+        <v>3126</v>
+      </c>
+      <c r="B1091" t="s">
+        <v>3130</v>
+      </c>
+      <c r="C1091">
+        <v>59855117</v>
+      </c>
+      <c r="D1091" s="11">
+        <f>ROUNDDOWN(C1091/2^16,0)</f>
+        <v>913</v>
+      </c>
+      <c r="E1091">
+        <f>ROUNDDOWN(C1091/2^14,0)</f>
+        <v>3653</v>
+      </c>
+    </row>
+    <row r="1092" spans="1:5">
+      <c r="A1092" t="s">
+        <v>3128</v>
+      </c>
+      <c r="C1092">
+        <f>C1090/C1091</f>
+        <v>2.1464196619981547E-2</v>
+      </c>
+      <c r="D1092">
+        <f>D1090/D1091</f>
+        <v>2.0810514786418401E-2</v>
+      </c>
+      <c r="E1092">
+        <f>E1090/E1091</f>
+        <v>2.1352313167259787E-2</v>
+      </c>
+    </row>
+    <row r="1093" spans="1:5">
+      <c r="B1093" t="s">
+        <v>3136</v>
+      </c>
+      <c r="C1093">
+        <f>ROUNDDOWN(C1092/C1096,0)</f>
+        <v>1</v>
+      </c>
+      <c r="D1093">
+        <f t="shared" ref="D1093:E1093" si="8">ROUNDDOWN(D1092/D1096,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E1093">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1096" spans="1:5">
+      <c r="B1096" t="s">
+        <v>3133</v>
+      </c>
+      <c r="C1096">
+        <f>1/2^6</f>
+        <v>1.5625E-2</v>
+      </c>
+      <c r="D1096">
+        <f t="shared" ref="D1096:E1096" si="9">1/2^6</f>
+        <v>1.5625E-2</v>
+      </c>
+      <c r="E1096">
+        <f t="shared" si="9"/>
+        <v>1.5625E-2</v>
+      </c>
+    </row>
+    <row r="1097" spans="1:5">
+      <c r="B1097" t="s">
         <v>3135</v>
       </c>
     </row>

</xml_diff>

<commit_message>
2025.11.21 pass part2-2 87 pat
</commit_message>
<xml_diff>
--- a/HW5/Softmax_table.xlsx
+++ b/HW5/Softmax_table.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c1d8b65b6adf7979/桌面/Github File/IC_Design_Laboratory/HW5/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jesse\OneDrive\桌面\Github File\IC_Design_Laboratory\HW5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="518" documentId="11_1B85D0BDD370594FA3B82111595ED87656CB84C1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6B320B9E-173E-4FED-B3E4-F279406CC2FE}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8C7EDB0-20DF-40A0-8151-8FE3E2386A5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3168" uniqueCount="3137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3181" uniqueCount="3139">
   <si>
     <t>Fixed-point Input (4Q6)</t>
   </si>
@@ -9506,6 +9506,14 @@
   </si>
   <si>
     <t>除法器輸出值</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>8-bit fraction</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>10-bit fraction</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -9687,10 +9695,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9978,7 +9982,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H1097"/>
+  <dimension ref="A1:H1107"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="25.19921875" bestFit="1" customWidth="1"/>
@@ -9987,7 +9991,7 @@
     <col min="4" max="4" width="27.8984375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="29.3984375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.8984375" customWidth="1"/>
-    <col min="7" max="7" width="49.8984375" customWidth="1"/>
+    <col min="7" max="7" width="27.69921875" customWidth="1"/>
     <col min="8" max="8" width="11.3984375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.69921875" bestFit="1" customWidth="1"/>
   </cols>
@@ -28165,7 +28169,7 @@
         <v>3135</v>
       </c>
     </row>
-    <row r="1089" spans="1:5">
+    <row r="1089" spans="1:7">
       <c r="C1089" t="s">
         <v>3132</v>
       </c>
@@ -28176,7 +28180,7 @@
         <v>3134</v>
       </c>
     </row>
-    <row r="1090" spans="1:5">
+    <row r="1090" spans="1:7">
       <c r="A1090" t="s">
         <v>3127</v>
       </c>
@@ -28195,7 +28199,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="1091" spans="1:5">
+    <row r="1091" spans="1:7">
       <c r="A1091" t="s">
         <v>3126</v>
       </c>
@@ -28214,7 +28218,7 @@
         <v>3653</v>
       </c>
     </row>
-    <row r="1092" spans="1:5">
+    <row r="1092" spans="1:7">
       <c r="A1092" t="s">
         <v>3128</v>
       </c>
@@ -28231,7 +28235,7 @@
         <v>2.1352313167259787E-2</v>
       </c>
     </row>
-    <row r="1093" spans="1:5">
+    <row r="1093" spans="1:7">
       <c r="B1093" t="s">
         <v>3136</v>
       </c>
@@ -28248,7 +28252,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="1096" spans="1:5">
+    <row r="1096" spans="1:7">
       <c r="B1096" t="s">
         <v>3133</v>
       </c>
@@ -28265,8 +28269,159 @@
         <v>1.5625E-2</v>
       </c>
     </row>
-    <row r="1097" spans="1:5">
+    <row r="1097" spans="1:7">
       <c r="B1097" t="s">
+        <v>3135</v>
+      </c>
+    </row>
+    <row r="1099" spans="1:7">
+      <c r="C1099" t="s">
+        <v>3132</v>
+      </c>
+      <c r="D1099" t="s">
+        <v>3131</v>
+      </c>
+      <c r="E1099" t="s">
+        <v>3134</v>
+      </c>
+      <c r="F1099" t="s">
+        <v>3137</v>
+      </c>
+      <c r="G1099" t="s">
+        <v>3138</v>
+      </c>
+    </row>
+    <row r="1100" spans="1:7">
+      <c r="A1100" t="s">
+        <v>3127</v>
+      </c>
+      <c r="B1100" t="s">
+        <v>3129</v>
+      </c>
+      <c r="C1100">
+        <v>969774</v>
+      </c>
+      <c r="D1100" s="11">
+        <f>ROUNDDOWN(C1100/2^16,0)</f>
+        <v>14</v>
+      </c>
+      <c r="E1100">
+        <f>ROUNDDOWN(C1100/2^14,0)</f>
+        <v>59</v>
+      </c>
+      <c r="F1100">
+        <f>ROUNDDOWN(C1100/2^12,0)</f>
+        <v>236</v>
+      </c>
+      <c r="G1100">
+        <f>ROUNDDOWN(C1100/2^10,0)</f>
+        <v>947</v>
+      </c>
+    </row>
+    <row r="1101" spans="1:7">
+      <c r="A1101" t="s">
+        <v>3126</v>
+      </c>
+      <c r="B1101" t="s">
+        <v>3130</v>
+      </c>
+      <c r="C1101">
+        <v>61952269</v>
+      </c>
+      <c r="D1101" s="11">
+        <f>ROUNDDOWN(C1101/2^16,0)</f>
+        <v>945</v>
+      </c>
+      <c r="E1101">
+        <f>ROUNDDOWN(C1101/2^14,0)</f>
+        <v>3781</v>
+      </c>
+      <c r="F1101">
+        <f>ROUNDDOWN(C1101/2^12,0)</f>
+        <v>15125</v>
+      </c>
+      <c r="G1101">
+        <f>ROUNDDOWN(C1101/2^10,0)</f>
+        <v>60500</v>
+      </c>
+    </row>
+    <row r="1102" spans="1:7">
+      <c r="A1102" t="s">
+        <v>3128</v>
+      </c>
+      <c r="C1102">
+        <f>C1100/C1101</f>
+        <v>1.5653567103409885E-2</v>
+      </c>
+      <c r="D1102">
+        <f>D1100/D1101</f>
+        <v>1.4814814814814815E-2</v>
+      </c>
+      <c r="E1102">
+        <f>E1100/E1101</f>
+        <v>1.5604337476857974E-2</v>
+      </c>
+      <c r="F1102">
+        <f>F1100/F1101</f>
+        <v>1.5603305785123967E-2</v>
+      </c>
+      <c r="G1102">
+        <f>G1100/G1101</f>
+        <v>1.5652892561983472E-2</v>
+      </c>
+    </row>
+    <row r="1103" spans="1:7">
+      <c r="B1103" t="s">
+        <v>3136</v>
+      </c>
+      <c r="C1103">
+        <f>ROUNDDOWN(C1102/C1106,0)</f>
+        <v>1</v>
+      </c>
+      <c r="D1103">
+        <f t="shared" ref="D1103:G1103" si="10">ROUNDDOWN(D1102/D1106,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E1103">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="F1103">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="G1103">
+        <f t="shared" si="10"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1106" spans="2:7">
+      <c r="B1106" t="s">
+        <v>3133</v>
+      </c>
+      <c r="C1106">
+        <f>1/2^6</f>
+        <v>1.5625E-2</v>
+      </c>
+      <c r="D1106">
+        <f t="shared" ref="D1106:G1106" si="11">1/2^6</f>
+        <v>1.5625E-2</v>
+      </c>
+      <c r="E1106">
+        <f t="shared" si="11"/>
+        <v>1.5625E-2</v>
+      </c>
+      <c r="F1106">
+        <f t="shared" si="11"/>
+        <v>1.5625E-2</v>
+      </c>
+      <c r="G1106">
+        <f t="shared" si="11"/>
+        <v>1.5625E-2</v>
+      </c>
+    </row>
+    <row r="1107" spans="2:7">
+      <c r="B1107" t="s">
         <v>3135</v>
       </c>
     </row>

</xml_diff>

<commit_message>
2025.11.21 fix syn error, area=22w, time=4ns
</commit_message>
<xml_diff>
--- a/HW5/Softmax_table.xlsx
+++ b/HW5/Softmax_table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jesse\OneDrive\桌面\Github File\IC_Design_Laboratory\HW5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8C7EDB0-20DF-40A0-8151-8FE3E2386A5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{234ED1BE-6AC9-4BD7-9BD3-EDB688D6193B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3181" uniqueCount="3139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3195" uniqueCount="3140">
   <si>
     <t>Fixed-point Input (4Q6)</t>
   </si>
@@ -9514,6 +9514,10 @@
   </si>
   <si>
     <t>10-bit fraction</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>12-bit fraction</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -9982,7 +9986,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H1107"/>
+  <dimension ref="A1:H1117"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="25.19921875" bestFit="1" customWidth="1"/>
@@ -9992,7 +9996,7 @@
     <col min="5" max="5" width="29.3984375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.8984375" customWidth="1"/>
     <col min="7" max="7" width="27.69921875" customWidth="1"/>
-    <col min="8" max="8" width="11.3984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.19921875" customWidth="1"/>
     <col min="9" max="9" width="9.69921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -28395,7 +28399,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="1106" spans="2:7">
+    <row r="1106" spans="1:8">
       <c r="B1106" t="s">
         <v>3133</v>
       </c>
@@ -28420,8 +28424,182 @@
         <v>1.5625E-2</v>
       </c>
     </row>
-    <row r="1107" spans="2:7">
+    <row r="1107" spans="1:8">
       <c r="B1107" t="s">
+        <v>3135</v>
+      </c>
+    </row>
+    <row r="1109" spans="1:8">
+      <c r="C1109" t="s">
+        <v>3132</v>
+      </c>
+      <c r="D1109" t="s">
+        <v>3131</v>
+      </c>
+      <c r="E1109" t="s">
+        <v>3134</v>
+      </c>
+      <c r="F1109" t="s">
+        <v>3137</v>
+      </c>
+      <c r="G1109" t="s">
+        <v>3138</v>
+      </c>
+      <c r="H1109" t="s">
+        <v>3139</v>
+      </c>
+    </row>
+    <row r="1110" spans="1:8">
+      <c r="A1110" t="s">
+        <v>3127</v>
+      </c>
+      <c r="B1110" t="s">
+        <v>3129</v>
+      </c>
+      <c r="C1110">
+        <v>1346398</v>
+      </c>
+      <c r="D1110" s="11">
+        <f>ROUNDDOWN(C1110/2^16,0)</f>
+        <v>20</v>
+      </c>
+      <c r="E1110">
+        <f>ROUNDDOWN(C1110/2^14,0)</f>
+        <v>82</v>
+      </c>
+      <c r="F1110">
+        <f>ROUNDDOWN(C1110/2^12,0)</f>
+        <v>328</v>
+      </c>
+      <c r="G1110">
+        <f>ROUNDDOWN(C1110/2^10,0)</f>
+        <v>1314</v>
+      </c>
+      <c r="H1110">
+        <f>ROUNDDOWN(C1110/2^8,0)</f>
+        <v>5259</v>
+      </c>
+    </row>
+    <row r="1111" spans="1:8">
+      <c r="A1111" t="s">
+        <v>3126</v>
+      </c>
+      <c r="B1111" t="s">
+        <v>3130</v>
+      </c>
+      <c r="C1111">
+        <v>86141170</v>
+      </c>
+      <c r="D1111" s="11">
+        <f>ROUNDDOWN(C1111/2^16,0)</f>
+        <v>1314</v>
+      </c>
+      <c r="E1111">
+        <f>ROUNDDOWN(C1111/2^14,0)</f>
+        <v>5257</v>
+      </c>
+      <c r="F1111">
+        <f>ROUNDDOWN(C1111/2^12,0)</f>
+        <v>21030</v>
+      </c>
+      <c r="G1111">
+        <f>ROUNDDOWN(C1111/2^10,0)</f>
+        <v>84122</v>
+      </c>
+      <c r="H1111">
+        <f>ROUNDDOWN(C1111/2^8,0)</f>
+        <v>336488</v>
+      </c>
+    </row>
+    <row r="1112" spans="1:8">
+      <c r="A1112" t="s">
+        <v>3128</v>
+      </c>
+      <c r="C1112">
+        <f>C1110/C1111</f>
+        <v>1.5630133651539677E-2</v>
+      </c>
+      <c r="D1112">
+        <f>D1110/D1111</f>
+        <v>1.5220700152207001E-2</v>
+      </c>
+      <c r="E1112">
+        <f>E1110/E1111</f>
+        <v>1.5598249952444359E-2</v>
+      </c>
+      <c r="F1112">
+        <f>F1110/F1111</f>
+        <v>1.5596766524013315E-2</v>
+      </c>
+      <c r="G1112">
+        <f>G1110/G1111</f>
+        <v>1.5620170704453056E-2</v>
+      </c>
+      <c r="H1112">
+        <f>H1110/H1111</f>
+        <v>1.562908632700126E-2</v>
+      </c>
+    </row>
+    <row r="1113" spans="1:8">
+      <c r="B1113" t="s">
+        <v>3136</v>
+      </c>
+      <c r="C1113">
+        <f>ROUNDDOWN(C1112/C1116,0)</f>
+        <v>1</v>
+      </c>
+      <c r="D1113">
+        <f t="shared" ref="D1113:H1113" si="12">ROUNDDOWN(D1112/D1116,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E1113">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="F1113">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="G1113">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="H1113">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1116" spans="1:8">
+      <c r="B1116" t="s">
+        <v>3133</v>
+      </c>
+      <c r="C1116">
+        <f>1/2^6</f>
+        <v>1.5625E-2</v>
+      </c>
+      <c r="D1116">
+        <f t="shared" ref="D1116:H1116" si="13">1/2^6</f>
+        <v>1.5625E-2</v>
+      </c>
+      <c r="E1116">
+        <f t="shared" si="13"/>
+        <v>1.5625E-2</v>
+      </c>
+      <c r="F1116">
+        <f t="shared" si="13"/>
+        <v>1.5625E-2</v>
+      </c>
+      <c r="G1116">
+        <f t="shared" si="13"/>
+        <v>1.5625E-2</v>
+      </c>
+      <c r="H1116">
+        <f t="shared" si="13"/>
+        <v>1.5625E-2</v>
+      </c>
+    </row>
+    <row r="1117" spans="1:8">
+      <c r="B1117" t="s">
         <v>3135</v>
       </c>
     </row>

</xml_diff>

<commit_message>
2025.11.21 all pass part2-2
</commit_message>
<xml_diff>
--- a/HW5/Softmax_table.xlsx
+++ b/HW5/Softmax_table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jesse\OneDrive\桌面\Github File\IC_Design_Laboratory\HW5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{234ED1BE-6AC9-4BD7-9BD3-EDB688D6193B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86FB99B9-91E9-4E4D-8902-CEFA3EB5F2A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3195" uniqueCount="3140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3225" uniqueCount="3144">
   <si>
     <t>Fixed-point Input (4Q6)</t>
   </si>
@@ -9518,6 +9518,22 @@
   </si>
   <si>
     <t>12-bit fraction</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>pat60</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>pat62</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>pat93</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>14-bit fraction</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -9986,7 +10002,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H1117"/>
+  <dimension ref="A1:I1136"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="25.19921875" bestFit="1" customWidth="1"/>
@@ -9997,7 +10013,7 @@
     <col min="6" max="6" width="15.8984375" customWidth="1"/>
     <col min="7" max="7" width="27.69921875" customWidth="1"/>
     <col min="8" max="8" width="19.19921875" customWidth="1"/>
-    <col min="9" max="9" width="9.69921875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.69921875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -28429,6 +28445,11 @@
         <v>3135</v>
       </c>
     </row>
+    <row r="1108" spans="1:8">
+      <c r="A1108" t="s">
+        <v>3140</v>
+      </c>
+    </row>
     <row r="1109" spans="1:8">
       <c r="C1109" t="s">
         <v>3132</v>
@@ -28516,27 +28537,27 @@
         <v>3128</v>
       </c>
       <c r="C1112">
-        <f>C1110/C1111</f>
+        <f t="shared" ref="C1112:H1112" si="12">C1110/C1111</f>
         <v>1.5630133651539677E-2</v>
       </c>
       <c r="D1112">
-        <f>D1110/D1111</f>
+        <f t="shared" si="12"/>
         <v>1.5220700152207001E-2</v>
       </c>
       <c r="E1112">
-        <f>E1110/E1111</f>
+        <f t="shared" si="12"/>
         <v>1.5598249952444359E-2</v>
       </c>
       <c r="F1112">
-        <f>F1110/F1111</f>
+        <f t="shared" si="12"/>
         <v>1.5596766524013315E-2</v>
       </c>
       <c r="G1112">
-        <f>G1110/G1111</f>
+        <f t="shared" si="12"/>
         <v>1.5620170704453056E-2</v>
       </c>
       <c r="H1112">
-        <f>H1110/H1111</f>
+        <f t="shared" si="12"/>
         <v>1.562908632700126E-2</v>
       </c>
     </row>
@@ -28549,23 +28570,23 @@
         <v>1</v>
       </c>
       <c r="D1113">
-        <f t="shared" ref="D1113:H1113" si="12">ROUNDDOWN(D1112/D1116,0)</f>
+        <f t="shared" ref="D1113:H1113" si="13">ROUNDDOWN(D1112/D1116,0)</f>
         <v>0</v>
       </c>
       <c r="E1113">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="F1113">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="G1113">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="H1113">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
     </row>
@@ -28578,29 +28599,400 @@
         <v>1.5625E-2</v>
       </c>
       <c r="D1116">
-        <f t="shared" ref="D1116:H1116" si="13">1/2^6</f>
+        <f t="shared" ref="D1116:H1116" si="14">1/2^6</f>
         <v>1.5625E-2</v>
       </c>
       <c r="E1116">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>1.5625E-2</v>
       </c>
       <c r="F1116">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>1.5625E-2</v>
       </c>
       <c r="G1116">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>1.5625E-2</v>
       </c>
       <c r="H1116">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>1.5625E-2</v>
       </c>
     </row>
     <row r="1117" spans="1:8">
       <c r="B1117" t="s">
         <v>3135</v>
+      </c>
+    </row>
+    <row r="1119" spans="1:8">
+      <c r="A1119" t="s">
+        <v>3141</v>
+      </c>
+    </row>
+    <row r="1120" spans="1:8">
+      <c r="C1120" t="s">
+        <v>3132</v>
+      </c>
+      <c r="D1120" t="s">
+        <v>3131</v>
+      </c>
+      <c r="E1120" t="s">
+        <v>3134</v>
+      </c>
+      <c r="F1120" t="s">
+        <v>3137</v>
+      </c>
+      <c r="G1120" t="s">
+        <v>3138</v>
+      </c>
+      <c r="H1120" t="s">
+        <v>3139</v>
+      </c>
+    </row>
+    <row r="1121" spans="1:9">
+      <c r="A1121" t="s">
+        <v>3127</v>
+      </c>
+      <c r="B1121" t="s">
+        <v>3129</v>
+      </c>
+      <c r="C1121">
+        <v>1811776</v>
+      </c>
+      <c r="D1121" s="11">
+        <f>ROUNDDOWN(C1121/2^16,0)</f>
+        <v>27</v>
+      </c>
+      <c r="E1121">
+        <f>ROUNDDOWN(C1121/2^14,0)</f>
+        <v>110</v>
+      </c>
+      <c r="F1121">
+        <f>ROUNDDOWN(C1121/2^12,0)</f>
+        <v>442</v>
+      </c>
+      <c r="G1121">
+        <f>ROUNDDOWN(C1121/2^10,0)</f>
+        <v>1769</v>
+      </c>
+      <c r="H1121">
+        <f>ROUNDDOWN(C1121/2^8,0)</f>
+        <v>7077</v>
+      </c>
+    </row>
+    <row r="1122" spans="1:9">
+      <c r="A1122" t="s">
+        <v>3126</v>
+      </c>
+      <c r="B1122" t="s">
+        <v>3130</v>
+      </c>
+      <c r="C1122">
+        <v>57974990</v>
+      </c>
+      <c r="D1122" s="11">
+        <f>ROUNDDOWN(C1122/2^16,0)</f>
+        <v>884</v>
+      </c>
+      <c r="E1122">
+        <f>ROUNDDOWN(C1122/2^14,0)</f>
+        <v>3538</v>
+      </c>
+      <c r="F1122">
+        <f>ROUNDDOWN(C1122/2^12,0)</f>
+        <v>14154</v>
+      </c>
+      <c r="G1122">
+        <f>ROUNDDOWN(C1122/2^10,0)</f>
+        <v>56616</v>
+      </c>
+      <c r="H1122">
+        <f>ROUNDDOWN(C1122/2^8,0)</f>
+        <v>226464</v>
+      </c>
+    </row>
+    <row r="1123" spans="1:9">
+      <c r="A1123" t="s">
+        <v>3128</v>
+      </c>
+      <c r="C1123">
+        <f t="shared" ref="C1123" si="15">C1121/C1122</f>
+        <v>3.1250992885035425E-2</v>
+      </c>
+      <c r="D1123">
+        <f t="shared" ref="D1123" si="16">D1121/D1122</f>
+        <v>3.0542986425339366E-2</v>
+      </c>
+      <c r="E1123">
+        <f t="shared" ref="E1123" si="17">E1121/E1122</f>
+        <v>3.1091011871113624E-2</v>
+      </c>
+      <c r="F1123">
+        <f t="shared" ref="F1123" si="18">F1121/F1122</f>
+        <v>3.1227921435636571E-2</v>
+      </c>
+      <c r="G1123">
+        <f t="shared" ref="G1123" si="19">G1121/G1122</f>
+        <v>3.1245584287127315E-2</v>
+      </c>
+      <c r="H1123">
+        <f t="shared" ref="H1123" si="20">H1121/H1122</f>
+        <v>3.125E-2</v>
+      </c>
+    </row>
+    <row r="1124" spans="1:9">
+      <c r="B1124" t="s">
+        <v>3136</v>
+      </c>
+      <c r="C1124">
+        <f>ROUNDDOWN(C1123/C1127,0)</f>
+        <v>2</v>
+      </c>
+      <c r="D1124">
+        <f t="shared" ref="D1124:H1124" si="21">ROUNDDOWN(D1123/D1127,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E1124">
+        <f t="shared" si="21"/>
+        <v>1</v>
+      </c>
+      <c r="F1124">
+        <f t="shared" si="21"/>
+        <v>1</v>
+      </c>
+      <c r="G1124">
+        <f t="shared" si="21"/>
+        <v>1</v>
+      </c>
+      <c r="H1124">
+        <f t="shared" si="21"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1127" spans="1:9">
+      <c r="B1127" t="s">
+        <v>3133</v>
+      </c>
+      <c r="C1127">
+        <f>1/2^6</f>
+        <v>1.5625E-2</v>
+      </c>
+      <c r="D1127">
+        <f t="shared" ref="D1127:H1127" si="22">1/2^6</f>
+        <v>1.5625E-2</v>
+      </c>
+      <c r="E1127">
+        <f t="shared" si="22"/>
+        <v>1.5625E-2</v>
+      </c>
+      <c r="F1127">
+        <f t="shared" si="22"/>
+        <v>1.5625E-2</v>
+      </c>
+      <c r="G1127">
+        <f t="shared" si="22"/>
+        <v>1.5625E-2</v>
+      </c>
+      <c r="H1127">
+        <f t="shared" si="22"/>
+        <v>1.5625E-2</v>
+      </c>
+    </row>
+    <row r="1128" spans="1:9">
+      <c r="A1128" t="s">
+        <v>3142</v>
+      </c>
+    </row>
+    <row r="1129" spans="1:9">
+      <c r="C1129" t="s">
+        <v>3132</v>
+      </c>
+      <c r="D1129" t="s">
+        <v>3131</v>
+      </c>
+      <c r="E1129" t="s">
+        <v>3134</v>
+      </c>
+      <c r="F1129" t="s">
+        <v>3137</v>
+      </c>
+      <c r="G1129" t="s">
+        <v>3138</v>
+      </c>
+      <c r="H1129" t="s">
+        <v>3139</v>
+      </c>
+      <c r="I1129" t="s">
+        <v>3143</v>
+      </c>
+    </row>
+    <row r="1130" spans="1:9">
+      <c r="A1130" t="s">
+        <v>3127</v>
+      </c>
+      <c r="B1130" t="s">
+        <v>3129</v>
+      </c>
+      <c r="C1130">
+        <v>4414669</v>
+      </c>
+      <c r="D1130" s="11">
+        <f>ROUNDDOWN(C1130/2^16,0)</f>
+        <v>67</v>
+      </c>
+      <c r="E1130">
+        <f>ROUNDDOWN(C1130/2^14,0)</f>
+        <v>269</v>
+      </c>
+      <c r="F1130">
+        <f>ROUNDDOWN(C1130/2^12,0)</f>
+        <v>1077</v>
+      </c>
+      <c r="G1130">
+        <f>ROUNDDOWN(C1130/2^10,0)</f>
+        <v>4311</v>
+      </c>
+      <c r="H1130">
+        <f>ROUNDDOWN(C1130/2^8,0)</f>
+        <v>17244</v>
+      </c>
+      <c r="I1130">
+        <f>ROUNDDOWN(C1130/2^6,0)</f>
+        <v>68979</v>
+      </c>
+    </row>
+    <row r="1131" spans="1:9">
+      <c r="A1131" t="s">
+        <v>3126</v>
+      </c>
+      <c r="B1131" t="s">
+        <v>3130</v>
+      </c>
+      <c r="C1131">
+        <v>282532440</v>
+      </c>
+      <c r="D1131" s="11">
+        <f>ROUNDDOWN(C1131/2^16,0)</f>
+        <v>4311</v>
+      </c>
+      <c r="E1131">
+        <f>ROUNDDOWN(C1131/2^14,0)</f>
+        <v>17244</v>
+      </c>
+      <c r="F1131">
+        <f>ROUNDDOWN(C1131/2^12,0)</f>
+        <v>68977</v>
+      </c>
+      <c r="G1131">
+        <f>ROUNDDOWN(C1131/2^10,0)</f>
+        <v>275910</v>
+      </c>
+      <c r="H1131">
+        <f>ROUNDDOWN(C1131/2^8,0)</f>
+        <v>1103642</v>
+      </c>
+      <c r="I1131">
+        <f>ROUNDDOWN(C1131/2^6,0)</f>
+        <v>4414569</v>
+      </c>
+    </row>
+    <row r="1132" spans="1:9">
+      <c r="A1132" t="s">
+        <v>3128</v>
+      </c>
+      <c r="C1132">
+        <f t="shared" ref="C1132" si="23">C1130/C1131</f>
+        <v>1.5625352614375893E-2</v>
+      </c>
+      <c r="D1132">
+        <f t="shared" ref="D1132" si="24">D1130/D1131</f>
+        <v>1.5541637671073997E-2</v>
+      </c>
+      <c r="E1132">
+        <f t="shared" ref="E1132" si="25">E1130/E1131</f>
+        <v>1.5599628856413824E-2</v>
+      </c>
+      <c r="F1132">
+        <f t="shared" ref="F1132" si="26">F1130/F1131</f>
+        <v>1.5613900285602448E-2</v>
+      </c>
+      <c r="G1132">
+        <f t="shared" ref="G1132" si="27">G1130/G1131</f>
+        <v>1.5624660215287594E-2</v>
+      </c>
+      <c r="H1132">
+        <f t="shared" ref="H1132:I1132" si="28">H1130/H1131</f>
+        <v>1.5624631900561958E-2</v>
+      </c>
+      <c r="I1132">
+        <f t="shared" si="28"/>
+        <v>1.5625307929267841E-2</v>
+      </c>
+    </row>
+    <row r="1133" spans="1:9">
+      <c r="B1133" t="s">
+        <v>3136</v>
+      </c>
+      <c r="C1133">
+        <f>ROUNDDOWN(C1132/C1136,0)</f>
+        <v>1</v>
+      </c>
+      <c r="D1133">
+        <f t="shared" ref="D1133:I1133" si="29">ROUNDDOWN(D1132/D1136,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E1133">
+        <f t="shared" si="29"/>
+        <v>0</v>
+      </c>
+      <c r="F1133">
+        <f t="shared" si="29"/>
+        <v>0</v>
+      </c>
+      <c r="G1133">
+        <f t="shared" si="29"/>
+        <v>0</v>
+      </c>
+      <c r="H1133">
+        <f t="shared" si="29"/>
+        <v>0</v>
+      </c>
+      <c r="I1133">
+        <f t="shared" si="29"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1136" spans="1:9">
+      <c r="B1136" t="s">
+        <v>3133</v>
+      </c>
+      <c r="C1136">
+        <f>1/2^6</f>
+        <v>1.5625E-2</v>
+      </c>
+      <c r="D1136">
+        <f t="shared" ref="D1136:I1136" si="30">1/2^6</f>
+        <v>1.5625E-2</v>
+      </c>
+      <c r="E1136">
+        <f t="shared" si="30"/>
+        <v>1.5625E-2</v>
+      </c>
+      <c r="F1136">
+        <f t="shared" si="30"/>
+        <v>1.5625E-2</v>
+      </c>
+      <c r="G1136">
+        <f t="shared" si="30"/>
+        <v>1.5625E-2</v>
+      </c>
+      <c r="H1136">
+        <f t="shared" si="30"/>
+        <v>1.5625E-2</v>
+      </c>
+      <c r="I1136">
+        <f t="shared" si="30"/>
+        <v>1.5625E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
2025.11.22 part2-2 syn area=28w time=4.4ns
</commit_message>
<xml_diff>
--- a/HW5/Softmax_table.xlsx
+++ b/HW5/Softmax_table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jesse\OneDrive\桌面\Github File\IC_Design_Laboratory\HW5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86FB99B9-91E9-4E4D-8902-CEFA3EB5F2A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03C55829-4BB6-483F-A273-652FCA2F6947}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3225" uniqueCount="3144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3246" uniqueCount="3165">
   <si>
     <t>Fixed-point Input (4Q6)</t>
   </si>
@@ -9534,6 +9534,90 @@
   </si>
   <si>
     <t>14-bit fraction</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>sofftV</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>token24</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>token32</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>token33</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>token40</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>token41</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>token43</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>token48</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>token50</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>token51</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>token53</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>token54</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>token55</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>token56</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>token57</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>token58</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>token59</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>token60</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>token61</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>token62</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>token63</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -10002,7 +10086,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I1136"/>
+  <dimension ref="A1:I1213"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="25.19921875" bestFit="1" customWidth="1"/>
@@ -28995,6 +29079,782 @@
         <v>1.5625E-2</v>
       </c>
     </row>
+    <row r="1140" spans="1:4">
+      <c r="A1140" t="s">
+        <v>3144</v>
+      </c>
+    </row>
+    <row r="1141" spans="1:4">
+      <c r="A1141">
+        <v>0</v>
+      </c>
+      <c r="D1141">
+        <f>A1141*B1141</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1142" spans="1:4">
+      <c r="A1142">
+        <v>0</v>
+      </c>
+      <c r="D1142">
+        <f t="shared" ref="D1142:D1205" si="31">A1142*B1142</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1143" spans="1:4">
+      <c r="A1143">
+        <v>0</v>
+      </c>
+      <c r="D1143">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1144" spans="1:4">
+      <c r="A1144">
+        <v>0</v>
+      </c>
+      <c r="D1144">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1145" spans="1:4">
+      <c r="A1145">
+        <v>0</v>
+      </c>
+      <c r="D1145">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1146" spans="1:4">
+      <c r="A1146">
+        <v>0</v>
+      </c>
+      <c r="D1146">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1147" spans="1:4">
+      <c r="A1147">
+        <v>0</v>
+      </c>
+      <c r="D1147">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1148" spans="1:4">
+      <c r="A1148">
+        <v>0</v>
+      </c>
+      <c r="D1148">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1149" spans="1:4">
+      <c r="D1149">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1150" spans="1:4">
+      <c r="A1150">
+        <v>0</v>
+      </c>
+      <c r="B1150">
+        <v>-6</v>
+      </c>
+      <c r="D1150">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1151" spans="1:4">
+      <c r="A1151">
+        <v>0</v>
+      </c>
+      <c r="D1151">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1152" spans="1:4">
+      <c r="A1152">
+        <v>0</v>
+      </c>
+      <c r="D1152">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1153" spans="1:4">
+      <c r="A1153">
+        <v>0</v>
+      </c>
+      <c r="D1153">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1154" spans="1:4">
+      <c r="A1154">
+        <v>0</v>
+      </c>
+      <c r="D1154">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1155" spans="1:4">
+      <c r="A1155">
+        <v>1</v>
+      </c>
+      <c r="B1155">
+        <v>9</v>
+      </c>
+      <c r="D1155">
+        <f t="shared" si="31"/>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1156" spans="1:4">
+      <c r="A1156">
+        <v>0</v>
+      </c>
+      <c r="D1156">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1157" spans="1:4">
+      <c r="A1157">
+        <v>0</v>
+      </c>
+      <c r="D1157">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1158" spans="1:4">
+      <c r="D1158">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1159" spans="1:4">
+      <c r="A1159">
+        <v>0</v>
+      </c>
+      <c r="D1159">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1160" spans="1:4">
+      <c r="A1160">
+        <v>0</v>
+      </c>
+      <c r="D1160">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1161" spans="1:4">
+      <c r="A1161">
+        <v>0</v>
+      </c>
+      <c r="D1161">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1162" spans="1:4">
+      <c r="A1162">
+        <v>0</v>
+      </c>
+      <c r="D1162">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1163" spans="1:4">
+      <c r="A1163">
+        <v>0</v>
+      </c>
+      <c r="D1163">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1164" spans="1:4">
+      <c r="A1164">
+        <v>0</v>
+      </c>
+      <c r="D1164">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1165" spans="1:4">
+      <c r="A1165">
+        <v>0</v>
+      </c>
+      <c r="D1165">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1166" spans="1:4">
+      <c r="A1166">
+        <v>0</v>
+      </c>
+      <c r="D1166">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1167" spans="1:4">
+      <c r="D1167">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1168" spans="1:4">
+      <c r="A1168">
+        <v>1</v>
+      </c>
+      <c r="B1168">
+        <v>3</v>
+      </c>
+      <c r="C1168" t="s">
+        <v>3145</v>
+      </c>
+      <c r="D1168">
+        <f t="shared" si="31"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1169" spans="1:4">
+      <c r="A1169">
+        <v>0</v>
+      </c>
+      <c r="B1169">
+        <v>17</v>
+      </c>
+      <c r="D1169">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1170" spans="1:4">
+      <c r="A1170">
+        <v>0</v>
+      </c>
+      <c r="B1170">
+        <v>-12</v>
+      </c>
+      <c r="D1170">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1171" spans="1:4">
+      <c r="A1171">
+        <v>0</v>
+      </c>
+      <c r="B1171">
+        <v>36</v>
+      </c>
+      <c r="D1171">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1172" spans="1:4">
+      <c r="A1172">
+        <v>0</v>
+      </c>
+      <c r="B1172">
+        <v>-5</v>
+      </c>
+      <c r="D1172">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1173" spans="1:4">
+      <c r="A1173">
+        <v>1</v>
+      </c>
+      <c r="B1173">
+        <v>7</v>
+      </c>
+      <c r="D1173">
+        <f t="shared" si="31"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="1174" spans="1:4">
+      <c r="A1174">
+        <v>0</v>
+      </c>
+      <c r="B1174">
+        <v>-44</v>
+      </c>
+      <c r="D1174">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1175" spans="1:4">
+      <c r="A1175">
+        <v>0</v>
+      </c>
+      <c r="B1175">
+        <v>9</v>
+      </c>
+      <c r="D1175">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1176" spans="1:4">
+      <c r="D1176">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1177" spans="1:4">
+      <c r="A1177">
+        <v>1</v>
+      </c>
+      <c r="B1177">
+        <v>42</v>
+      </c>
+      <c r="C1177" t="s">
+        <v>3146</v>
+      </c>
+      <c r="D1177">
+        <f t="shared" si="31"/>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="1178" spans="1:4">
+      <c r="A1178">
+        <v>3</v>
+      </c>
+      <c r="B1178">
+        <v>-1</v>
+      </c>
+      <c r="C1178" t="s">
+        <v>3147</v>
+      </c>
+      <c r="D1178">
+        <f t="shared" si="31"/>
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="1179" spans="1:4">
+      <c r="A1179">
+        <v>0</v>
+      </c>
+      <c r="B1179">
+        <v>-2</v>
+      </c>
+      <c r="D1179">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1180" spans="1:4">
+      <c r="A1180">
+        <v>0</v>
+      </c>
+      <c r="D1180">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1181" spans="1:4">
+      <c r="A1181">
+        <v>0</v>
+      </c>
+      <c r="D1181">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1182" spans="1:4">
+      <c r="A1182">
+        <v>0</v>
+      </c>
+      <c r="D1182">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1183" spans="1:4">
+      <c r="A1183">
+        <v>0</v>
+      </c>
+      <c r="D1183">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1184" spans="1:4">
+      <c r="A1184">
+        <v>0</v>
+      </c>
+      <c r="D1184">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1185" spans="1:4">
+      <c r="D1185">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1186" spans="1:4">
+      <c r="A1186">
+        <v>0</v>
+      </c>
+      <c r="C1186" t="s">
+        <v>3148</v>
+      </c>
+      <c r="D1186">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1187" spans="1:4">
+      <c r="A1187">
+        <v>1</v>
+      </c>
+      <c r="B1187">
+        <v>-4</v>
+      </c>
+      <c r="C1187" t="s">
+        <v>3149</v>
+      </c>
+      <c r="D1187">
+        <f t="shared" si="31"/>
+        <v>-4</v>
+      </c>
+    </row>
+    <row r="1188" spans="1:4">
+      <c r="A1188">
+        <v>0</v>
+      </c>
+      <c r="D1188">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1189" spans="1:4">
+      <c r="A1189">
+        <v>1</v>
+      </c>
+      <c r="B1189">
+        <v>19</v>
+      </c>
+      <c r="C1189" t="s">
+        <v>3150</v>
+      </c>
+      <c r="D1189">
+        <f t="shared" si="31"/>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1190" spans="1:4">
+      <c r="A1190">
+        <v>0</v>
+      </c>
+      <c r="D1190">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1191" spans="1:4">
+      <c r="A1191">
+        <v>0</v>
+      </c>
+      <c r="D1191">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1192" spans="1:4">
+      <c r="A1192">
+        <v>0</v>
+      </c>
+      <c r="D1192">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1193" spans="1:4">
+      <c r="A1193">
+        <v>0</v>
+      </c>
+      <c r="D1193">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1194" spans="1:4">
+      <c r="D1194">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1195" spans="1:4">
+      <c r="A1195">
+        <v>2</v>
+      </c>
+      <c r="B1195">
+        <v>-2</v>
+      </c>
+      <c r="C1195" t="s">
+        <v>3151</v>
+      </c>
+      <c r="D1195">
+        <f t="shared" si="31"/>
+        <v>-4</v>
+      </c>
+    </row>
+    <row r="1196" spans="1:4">
+      <c r="A1196">
+        <v>0</v>
+      </c>
+      <c r="D1196">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1197" spans="1:4">
+      <c r="A1197">
+        <v>5</v>
+      </c>
+      <c r="B1197">
+        <v>-19</v>
+      </c>
+      <c r="C1197" t="s">
+        <v>3152</v>
+      </c>
+      <c r="D1197">
+        <f t="shared" si="31"/>
+        <v>-95</v>
+      </c>
+    </row>
+    <row r="1198" spans="1:4">
+      <c r="A1198">
+        <v>1</v>
+      </c>
+      <c r="B1198">
+        <v>-2</v>
+      </c>
+      <c r="C1198" t="s">
+        <v>3153</v>
+      </c>
+      <c r="D1198">
+        <f t="shared" si="31"/>
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="1199" spans="1:4">
+      <c r="A1199">
+        <v>0</v>
+      </c>
+      <c r="D1199">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1200" spans="1:4">
+      <c r="A1200">
+        <v>1</v>
+      </c>
+      <c r="B1200">
+        <v>-1</v>
+      </c>
+      <c r="C1200" t="s">
+        <v>3154</v>
+      </c>
+      <c r="D1200">
+        <f t="shared" si="31"/>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="1201" spans="1:4">
+      <c r="A1201">
+        <v>2</v>
+      </c>
+      <c r="B1201">
+        <v>-9</v>
+      </c>
+      <c r="C1201" t="s">
+        <v>3155</v>
+      </c>
+      <c r="D1201">
+        <f t="shared" si="31"/>
+        <v>-18</v>
+      </c>
+    </row>
+    <row r="1202" spans="1:4">
+      <c r="A1202">
+        <v>2</v>
+      </c>
+      <c r="B1202">
+        <v>-6</v>
+      </c>
+      <c r="C1202" t="s">
+        <v>3156</v>
+      </c>
+      <c r="D1202">
+        <f t="shared" si="31"/>
+        <v>-12</v>
+      </c>
+    </row>
+    <row r="1203" spans="1:4">
+      <c r="D1203">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1204" spans="1:4">
+      <c r="A1204">
+        <v>2</v>
+      </c>
+      <c r="B1204">
+        <v>-14</v>
+      </c>
+      <c r="C1204" t="s">
+        <v>3157</v>
+      </c>
+      <c r="D1204">
+        <f t="shared" si="31"/>
+        <v>-28</v>
+      </c>
+    </row>
+    <row r="1205" spans="1:4">
+      <c r="A1205">
+        <v>1</v>
+      </c>
+      <c r="B1205">
+        <v>-2</v>
+      </c>
+      <c r="C1205" t="s">
+        <v>3158</v>
+      </c>
+      <c r="D1205">
+        <f t="shared" si="31"/>
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="1206" spans="1:4">
+      <c r="A1206">
+        <v>2</v>
+      </c>
+      <c r="B1206">
+        <v>-18</v>
+      </c>
+      <c r="C1206" t="s">
+        <v>3159</v>
+      </c>
+      <c r="D1206">
+        <f t="shared" ref="D1206:D1211" si="32">A1206*B1206</f>
+        <v>-36</v>
+      </c>
+    </row>
+    <row r="1207" spans="1:4">
+      <c r="A1207">
+        <v>1</v>
+      </c>
+      <c r="B1207">
+        <v>-14</v>
+      </c>
+      <c r="C1207" t="s">
+        <v>3160</v>
+      </c>
+      <c r="D1207">
+        <f t="shared" si="32"/>
+        <v>-14</v>
+      </c>
+    </row>
+    <row r="1208" spans="1:4">
+      <c r="A1208">
+        <v>1</v>
+      </c>
+      <c r="B1208">
+        <v>-8</v>
+      </c>
+      <c r="C1208" t="s">
+        <v>3161</v>
+      </c>
+      <c r="D1208">
+        <f t="shared" si="32"/>
+        <v>-8</v>
+      </c>
+    </row>
+    <row r="1209" spans="1:4">
+      <c r="A1209">
+        <v>2</v>
+      </c>
+      <c r="B1209">
+        <v>-5</v>
+      </c>
+      <c r="C1209" t="s">
+        <v>3162</v>
+      </c>
+      <c r="D1209">
+        <f t="shared" si="32"/>
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="1210" spans="1:4">
+      <c r="A1210">
+        <v>1</v>
+      </c>
+      <c r="B1210">
+        <v>-5</v>
+      </c>
+      <c r="C1210" t="s">
+        <v>3163</v>
+      </c>
+      <c r="D1210">
+        <f t="shared" si="32"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="1211" spans="1:4">
+      <c r="A1211">
+        <v>2</v>
+      </c>
+      <c r="B1211">
+        <v>-1</v>
+      </c>
+      <c r="C1211" t="s">
+        <v>3164</v>
+      </c>
+      <c r="D1211">
+        <f t="shared" si="32"/>
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="1213" spans="1:4">
+      <c r="D1213">
+        <f>SUM(D1141:D1211)</f>
+        <v>-164</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1041:G1041"/>

</xml_diff>